<commit_message>
Separate crypto ticker universe
</commit_message>
<xml_diff>
--- a/validTickers/validtickers_IT_MIB30_with_sector.xlsx
+++ b/validTickers/validtickers_IT_MIB30_with_sector.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1453,74 +1453,6 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Etherium</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>ETH-USD</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Bitcoin</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>BTC-USD</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Solana</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>SOL-USD</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Cardano</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>ADA-USD</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>